<commit_message>
feat: expose all canonical pages in shared footer
</commit_message>
<xml_diff>
--- a/docs/UK-ETA_ページ管理一覧_2026-08-07.xlsx
+++ b/docs/UK-ETA_ページ管理一覧_2026-08-07.xlsx
@@ -986,11 +986,11 @@
         </is>
       </c>
       <c r="B8" s="32" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="C8" s="32" t="inlineStr">
         <is>
-          <t>ヘッダー、FAQメニュー、またはフッターから直接到達可能</t>
+          <t>全26正規ページが共通フッターから直接到達可能</t>
         </is>
       </c>
     </row>
@@ -1024,6 +1024,8 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="33" t="inlineStr">
         <is>
@@ -1127,6 +1129,8 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="33" t="inlineStr">
         <is>
@@ -1602,7 +1606,7 @@
       </c>
       <c r="H9" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I9" s="37" t="inlineStr">
@@ -1670,7 +1674,7 @@
       </c>
       <c r="H10" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I10" s="37" t="inlineStr">
@@ -1738,7 +1742,7 @@
       </c>
       <c r="H11" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I11" s="37" t="inlineStr">
@@ -1806,7 +1810,7 @@
       </c>
       <c r="H12" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I12" s="37" t="inlineStr">
@@ -1874,7 +1878,7 @@
       </c>
       <c r="H13" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I13" s="37" t="inlineStr">
@@ -1942,7 +1946,7 @@
       </c>
       <c r="H14" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I14" s="37" t="inlineStr">
@@ -2010,7 +2014,7 @@
       </c>
       <c r="H15" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I15" s="37" t="inlineStr">
@@ -2078,7 +2082,7 @@
       </c>
       <c r="H16" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I16" s="37" t="inlineStr">
@@ -2146,7 +2150,7 @@
       </c>
       <c r="H17" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I17" s="37" t="inlineStr">
@@ -2214,7 +2218,7 @@
       </c>
       <c r="H18" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I18" s="37" t="inlineStr">
@@ -2282,7 +2286,7 @@
       </c>
       <c r="H19" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I19" s="37" t="inlineStr">
@@ -2350,7 +2354,7 @@
       </c>
       <c r="H20" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I20" s="37" t="inlineStr">
@@ -2418,7 +2422,7 @@
       </c>
       <c r="H21" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I21" s="37" t="inlineStr">
@@ -2962,7 +2966,7 @@
       </c>
       <c r="H29" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I29" s="37" t="inlineStr">
@@ -3030,7 +3034,7 @@
       </c>
       <c r="H30" s="37" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>フッター</t>
         </is>
       </c>
       <c r="I30" s="37" t="inlineStr">

</xml_diff>